<commit_message>
Viva update and more testing feedback
</commit_message>
<xml_diff>
--- a/Project/Testing Results.xlsx
+++ b/Project/Testing Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\MA-Dissertation\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6389483-7F4C-422D-96BE-3E502EF8949E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19EAA4E-BFA1-4EC7-B224-6204993DEF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
   <si>
     <t>Tester</t>
   </si>
@@ -97,16 +97,57 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Ryan</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1x1g8LKJPQI3DvhubyJicdpeBLbwPIJFp?usp=sharing</t>
+  </si>
+  <si>
+    <t>No Difficulty, however could not find generator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Straight paths were main roads, different angle roads where usually secondary paths with no exit. </t>
+  </si>
+  <si>
+    <t>Size of paths</t>
+  </si>
+  <si>
+    <t>Ilumination</t>
+  </si>
+  <si>
+    <t>Landmarks 2</t>
+  </si>
+  <si>
+    <t>1min 98sec</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>Used the watertower to orient self as main guidence tool</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1x1g8LKJPQI3DvhubyJicdpeBLbwPIJFp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -224,10 +265,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -265,23 +307,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -560,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:M15"/>
+  <dimension ref="B2:N15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.88671875" customWidth="1"/>
@@ -577,7 +620,7 @@
     <col min="13" max="13" width="69.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -592,7 +635,7 @@
       </c>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>11</v>
       </c>
@@ -611,24 +654,24 @@
       <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="13" t="s">
         <v>5</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J3" s="5"/>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L3" s="13" t="s">
+      <c r="L3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="13" t="s">
+      <c r="M3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
@@ -648,17 +691,17 @@
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="5">
+      <c r="K4" s="3">
         <v>5</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
@@ -678,17 +721,17 @@
       </c>
       <c r="I5" s="10"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="5">
+      <c r="K5" s="3">
         <v>5</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="M5" s="15" t="s">
+      <c r="M5" s="16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:13" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:14" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
@@ -698,7 +741,7 @@
       <c r="D6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="14" t="s">
         <v>21</v>
       </c>
       <c r="F6" s="5"/>
@@ -708,69 +751,137 @@
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="5">
+      <c r="K6" s="3">
         <v>5</v>
       </c>
-      <c r="L6" s="16" t="s">
+      <c r="L6" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="M6" s="15" t="s">
+      <c r="M6" s="16" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B7" s="5"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="5"/>
+      <c r="N6" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="H7" s="6" t="s">
+        <v>22</v>
+      </c>
       <c r="I7" s="10"/>
       <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B8" s="5"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="5"/>
+      <c r="K7" s="3">
+        <v>5</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>8</v>
+      </c>
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="H8" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I8" s="10"/>
       <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B9" s="5"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="5"/>
+      <c r="K8" s="3">
+        <v>5</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="3">
+        <v>2</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>9</v>
+      </c>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="H9" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="I9" s="10"/>
       <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B10" s="5"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="K9" s="3">
+        <v>4</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="5">
+        <v>1</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I10" s="10"/>
       <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
+      <c r="K10" s="3"/>
       <c r="L10" s="5"/>
-    </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="M10" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="N10" s="15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B11" s="5"/>
       <c r="C11" s="3"/>
       <c r="D11" s="5"/>
@@ -780,10 +891,11 @@
       <c r="H11" s="5"/>
       <c r="I11" s="10"/>
       <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
+      <c r="K11" s="3"/>
       <c r="L11" s="5"/>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="M11" s="18"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B12" s="5"/>
       <c r="C12" s="3"/>
       <c r="D12" s="5"/>
@@ -793,10 +905,11 @@
       <c r="H12" s="5"/>
       <c r="I12" s="10"/>
       <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
+      <c r="K12" s="3"/>
       <c r="L12" s="5"/>
-    </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="M12" s="18"/>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B13" s="5"/>
       <c r="C13" s="3"/>
       <c r="D13" s="5"/>
@@ -806,10 +919,11 @@
       <c r="H13" s="5"/>
       <c r="I13" s="10"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
+      <c r="K13" s="3"/>
       <c r="L13" s="5"/>
-    </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="M13" s="18"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B14" s="5"/>
       <c r="C14" s="3"/>
       <c r="D14" s="5"/>
@@ -819,10 +933,11 @@
       <c r="H14" s="5"/>
       <c r="I14" s="10"/>
       <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
+      <c r="K14" s="3"/>
       <c r="L14" s="5"/>
-    </row>
-    <row r="15" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="M14" s="18"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
       <c r="C15" s="4"/>
       <c r="D15" s="11"/>
@@ -832,10 +947,15 @@
       <c r="H15" s="11"/>
       <c r="I15" s="12"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="19"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="N6" r:id="rId1" xr:uid="{EAC966FB-C271-4A91-A0F1-94FCFCAAE187}"/>
+    <hyperlink ref="N10" r:id="rId2" xr:uid="{452639ED-929B-478E-9568-DD03DCE8A86C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Viva Progress + Docs
</commit_message>
<xml_diff>
--- a/Project/Testing Results.xlsx
+++ b/Project/Testing Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\MA-Dissertation\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19EAA4E-BFA1-4EC7-B224-6204993DEF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BD21E2A-61F0-42F0-A401-6BDA0C92B2BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="1695" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="40">
   <si>
     <t>Tester</t>
   </si>
@@ -130,6 +130,22 @@
   </si>
   <si>
     <t>https://drive.google.com/drive/folders/1x1g8LKJPQI3DvhubyJicdpeBLbwPIJFp</t>
+  </si>
+  <si>
+    <t>Will</t>
+  </si>
+  <si>
+    <t>Julia</t>
+  </si>
+  <si>
+    <t>street lamps that were on and water towers</t>
+  </si>
+  <si>
+    <t>yes, in the landmark prototype, right when u spawn in. i took the left turn bc i couldn't see the water tower or anything from the spawn point, so i just gambled and it turned out to be the longer way</t>
+  </si>
+  <si>
+    <t>The genarator was very visablaus as well as the jump pad on the first level
+ And on the other 2 levels they guided me to the end to find the genarator</t>
   </si>
 </sst>
 </file>
@@ -269,7 +285,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -321,7 +337,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -603,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:N15"/>
+  <dimension ref="B2:N16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.88671875" customWidth="1"/>
@@ -872,7 +896,9 @@
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="5"/>
-      <c r="K10" s="3"/>
+      <c r="K10" s="3">
+        <v>5</v>
+      </c>
       <c r="L10" s="5"/>
       <c r="M10" s="18" t="s">
         <v>33</v>
@@ -882,74 +908,164 @@
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B11" s="5"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="B11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="9">
+        <v>5.4166666666666669E-2</v>
+      </c>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="H11" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I11" s="10"/>
       <c r="J11" s="5"/>
-      <c r="K11" s="3"/>
+      <c r="K11" s="3">
+        <v>5</v>
+      </c>
       <c r="L11" s="5"/>
       <c r="M11" s="18"/>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B12" s="5"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+    <row r="12" spans="2:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="3">
+        <v>3</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="9">
+        <v>1.8749999999999999E-2</v>
+      </c>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
+      <c r="H12" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I12" s="10"/>
       <c r="J12" s="5"/>
-      <c r="K12" s="3"/>
+      <c r="K12" s="3">
+        <v>5</v>
+      </c>
       <c r="L12" s="5"/>
-      <c r="M12" s="18"/>
+      <c r="M12" s="19" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B13" s="5"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="B13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="3">
+        <v>3</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="9">
+        <v>4.8611111111111112E-2</v>
+      </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
+      <c r="H13" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I13" s="10"/>
       <c r="J13" s="5"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="18"/>
+      <c r="K13" s="3">
+        <v>4</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M13" s="19"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B14" s="5"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="B14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="3">
+        <v>4</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="9">
+        <v>3.125E-2</v>
+      </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
+      <c r="H14" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I14" s="10"/>
       <c r="J14" s="5"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="5"/>
+      <c r="K14" s="3">
+        <v>4</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="M14" s="18"/>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B15" s="5"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
+    <row r="15" spans="2:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B15" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="3">
+        <v>4</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="9">
+        <v>1.3888888888888888E-2</v>
+      </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
+      <c r="H15" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I15" s="12"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="19"/>
+      <c r="K15" s="4">
+        <v>4</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M15" s="21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="3">
+        <v>4</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E16" s="9">
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="K16" s="20">
+        <v>4</v>
+      </c>
+      <c r="L16" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>